<commit_message>
docs: refresh CH v4 story sheet from live-wiring file (16 beats + branch)
Reflects current creator-house-v4.json: your D1-1/D1-3 rewrites, terrace secret,
Nominations, and the branching Elimination (⑂ variant row shows the shielded→Dev
path). Read-me flags the still-pending pieces (D3-2 reveal, gender-lock, screenshots).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/creator-house-v4-story.xlsx
+++ b/docs/creator-house-v4-story.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Story (v4 rewrite)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Story (v4 draft · live-wiring)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Characters" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Endings (2×2)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Read me" sheetId="4" state="visible" r:id="rId4"/>
@@ -432,31 +432,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:Q35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="5" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="44" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
     <col width="40" customWidth="1" min="14" max="14"/>
-    <col width="40" customWidth="1" min="15" max="15"/>
-    <col width="34" customWidth="1" min="16" max="16"/>
+    <col width="36" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="16" max="16"/>
+    <col width="32" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ch</t>
+          <t>Ch/Day</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -511,25 +512,30 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>Flag</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Outcome</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>DM (from → messages)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Post caption</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Post reactions</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>House reacts</t>
         </is>
@@ -556,14 +562,16 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Villa ka gate khulta hai. Andar music, ring lights, aur ek paani ka pool jo golden reflection maar raha hai. Do hafte pehle teri ek reel raat-o-raat viral ho gayi thi — aur ab tu yahaan hai.
-Char creators pehle se andar. Ria sofa pe, sunglasses lagaye, phone se nazar hataye bina. Zoya ne muskaan already load kar rakhi hai. Ananya aur Kabir ek doosre se kuch keh rahe the — ab dono chup.
-Sabki nazar ek saath tujh pe. Pehla impression sirf ek baar banta hai.</t>
+          <t>Gate ke us paar villa dhoop mein chamak raha hai. Tum andar kadam rakhte ho — aur ek pal ko ruk jaate ho. Aisa ghar tumne sirf feed pe scroll karte hue dekha tha.
+Lounge mein sab tham gaye. Ria tumhari Ananya se poochti hai —
+Ria: Yeh wahi hai na jiski reel viral ho gayi thi pichle mahine? 👀
+Ananya: Umm… haan. Haan, main isko jaanti hun.
+Ananya ki aankhein ek pal ke liye tumse mili — phir hat gayi. 3 saal ho gaye. Par woh nazar tumhe abhi bhi yaad hai.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Creator House mein pehla kadam kaise rakhta hai?</t>
+          <t>Kaise enter karte ho Creator House mein?</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -573,97 +581,99 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Bold entry — apni entrance reel post kar de</t>
+          <t>Quiet entry — observe first</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Camera on, energy loud. Sabko dikha de tu kyun trending tha. (fame +3, par ab sab expose)</t>
+          <t>Let the house come to you. (fame +1)</t>
         </is>
       </c>
       <c r="J2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>zoya → Chup-chaap wale? Interesting. Main aise logon ko jaldi padh leti hun. 😏 / Ek advice — is ghar mein har koi acting kar raha hai. Main tumhe bata sakti hun kaun kya chhupa raha hai. Baad mein baat karein? 💅</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>House Watch: naya contestant andar aaya aur seedha corner se sabko scan kar raha hai. the silent gameplayer arc? 👀 #CreatorHouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>D1-1</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Pehla Kadam</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Loud entry — sabka dhyan kheencho</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Confident, noisy, unforgettable. (fame +3)</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Post</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>Creator House unlocked. 🔥 Koi chupke se nahi aata — main toh bilkul nahi. Day 1, let's gooo. #CreatorHouse #Day1</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>Creator House unlocked. 🔥 Koi chupke se nahi aata — main toh bilkul nahi. Day 1, let’s gooo. #CreatorHouse #Day1</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>ria: Loud arrivals do do cheezein hoti hain — confidence ya overcompensation. Filing it away. 👑
 kabir: HAAN BHAI ye energy 😭🔥 welcome to the madhouse
 House Watch: day 1 ki entry hi itni loud?? this season is gonna be CHAOS 👀</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>ria: Kuch log aate hain. Kuch log entry maarte hain. Day 1 se hi volume max. Let's see kab tak chalti hai battery. 🤍</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Morning</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>D1-1</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Pehla Kadam</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Room read kar — pehle observe kar</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Bolna kam, dekhna zyada. Ghar ko tere paas aane de. (fame +1)</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>zoya → Chup-chaap wale? Interesting. Main aise logon ko jaldi padh leti hun. 😏 / Ek advice — is ghar mein har koi acting kar raha hai. Main tumhe bata sakti hun kaun kya chhupa raha hai. Baad mein baat karein? 💅</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr"/>
-      <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>House Watch: naya contestant andar aaya aur seedha corner se sabko scan kar raha hai. the silent gameplayer arc? 👀 #CreatorHouse</t>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>ria: Kuch log aate hain. Kuch log entry maarte hain. Day 1 se hi volume max. Let’s see kab tak chalti hai battery. 🤍</t>
         </is>
       </c>
     </row>
@@ -688,9 +698,11 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Dopahar ko ghar ka pehla content challenge drop hota hai — ek common trend, aur sawaal ek hi: sabse zyada views kaun laata hai. Golden light perfect hai.
-Ria seedhi khadi ho jaati hai, hair flip, aur announce kar deti hai jaise result already decide ho gaya: "Main pehle jaati hun. Bar set kar deti hun, phir tum log follow kar lena."
-Kabir tere kaan mein: "Bhai, iski energy match kar — ya iska pura format ulta parody maar de. Viral bhi, aur Ria ko jala bhi dega."</t>
+          <t>Ghar ke speakers pe pehla announcement. Pehla challenge — ek trend, ek winner. Jeeta toh followers, aur shayad season ki pehli badi brand deal. Sab apne phone utha chuke hain.
+Ria: Main pehle. Aisi cheezein experience se aati hain, sabke bas ki nahi. Baaki sab meri reel ke baad decide kar lena kya karna hai. 👑
+Ria ne bar itna upar rakh diya ki poora ghar ek second ke liye chup ho gaya. Yehi uska move hai — pehle bol do ki tum best ho, taaki sab tumse compare karein.
+Kabir: Bhai suno — do raaste. Ya iski energy match karke seedhi takkar, ya iska pura 'aesthetic morning routine' format ulta parody maar do. Funny, viral, aur Ria ka ego thoda hilega. 😏
+» Ria ne khud ko standard bana diya. Ya toh use aaine ki tarah dikha de, ya apni alag lane pakad le. Pehli reel — sab dekh rahe hain.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -721,25 +733,26 @@
           <t>ria −2</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>Post</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>POV: koi apni 'effortless aesthetic morning routine' ke liye 3 ghante set-up karta hai 💅✨ (parody hai relax 😂) #CreatorHouse #Day1</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>ria: Cute. Meri reel ke bina tumhare paas content bhi nahi tha. Main flattered hun. 👀
 zoya: OKAY not the day 1 shots being fired 💅 I'm obsessed, keep going babe
 House Watch: DAY 1 pe ria ka parody?? bhai brave hai ya paagal, decide nahi ho pa raha 😭</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="Q4" s="2" t="inlineStr">
         <is>
           <t>ria: Imitation flattery nahi hota jab tumhare paas apna kuch na ho. Day 1 se hi meri reel copy kar rahe hain. Main hun hi itni iconic. 🤍 #CreatorHouse</t>
         </is>
@@ -789,19 +802,20 @@
           <t>kabir +3</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>{ally} → Yaar tune Ria ko poora ignore kar diya aur apna banaya 😭 respect / Sabse easy tha uspe cheap shot maarna. Tune nahi maara. Tu apne dum pe khela. / Idhar sabko lagta hai main sirf jokes hun. Tu shayad pehla hai jisne kaam pe focus kiya, drama pe nahi. Ye yaad rahega. 🔥</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>kabir → Yaar tune Ria ko poora ignore kar diya aur apna banaya 😭 respect / Sabse easy tha uspe cheap shot maarna. Tune nahi maara. Tu apne dum pe khela. / Idhar sabko lagta hai main sirf jokes hun. Tu shayad pehla hai jisne kaam pe focus kiya, drama pe nahi. Ye yaad rahega. 🔥</t>
+        </is>
+      </c>
       <c r="O5" s="2" t="inlineStr"/>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr">
         <is>
           <t>Creator Tea: kisi ne ria ka bait poora ignore karke apni reel bana di. building a brand vs building beef — day 1 se hi clear ho gaya kaun kya hai 🍿</t>
         </is>
@@ -828,9 +842,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>1 baja hai. Ghar ka shor thand chuka hai, cameras andar so gaye hain. Tu terrace pe hai — pehli baar akele, pehli baar khulke saans le raha hai.
-Darwaaza halka sa khulta hai. Ananya. Do mug coffee, ek tere liye. Koi ring light nahi, koi audience nahi. Sirf sheher ki roshni door tak faili hui.
-Ananya railing pe tere bagal mein aa ke khada ho jaata hai. "Yahaan camera nahi hai," woh dheere se bolta hai. "Toh… tu sach mein kaisa hai?"</t>
+          <t>Raat ke 1 baje villa ekdum shaant hai. Neeche koi ring light nahi jal rahi, koi phone up nahi hai. Pehli baar tujhe lagta hai jaise tu perform nahi kar raha.
+Terrace ka darwaaza khulta hai. Ananya — haath mein do coffee mug. Din bhar sab in-front-of-camera version dekh rahe the. Ye wala Ananya alag hai. Guarded. Real.
+Ananya: Le, teri coffee. Main bhaag rahi thi neeche wale circus se. 😅 Din bhar sab apna 'content face' pehne ghoom rahe the… tera bhi wahi tha na? 🥺
+Ananya coffee ka sip leti hai aur door dekhne lagti hai. Phir dheere se — jaise ye sawaal kisi aur se nahi poochti — tere taraf mudti hai.
+Ananya: Idhar camera nahi hai. Followers nahi hain. Toh… sach batao. Tum sach mein kaise ho? ✨
+» Koi audience nahi. Sirf tu, woh, aur ye sawaal. Ise sach mein sunega — ya cool banke aage badh jaayega?</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -845,12 +862,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Khul ja — sach mein sun</t>
+          <t>Khul jaao, sach main suno</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Mask utaar de. Coffee, sach, aur ek adhoora sa kuch jo teen saal se hai. (crush +6, fame -1)</t>
+          <t>Mask utaar de. Coffee, sach, aur ek adhoora sa kuch jo teen saal se hai. (crush +6, fame −1)</t>
         </is>
       </c>
       <c r="J6" s="2" t="n">
@@ -861,19 +878,20 @@
           <t>ananya +6</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>{crush} → Tu ruk gaya. Sabse aasaan tha topic ghumaana, joke maar dena. Tune nahi kiya. 🥺 / Pata hai teen saal main sochta raha — agar us raat kuch alag hota toh? Aur ab tu yahaan khada hai, mere saamne, poori tarah real. / Aaj raat kisi ko mat batana. Ye wala tu… ye sirf mere liye tha. Good night. ✨</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>ananya → Tu ruk gaya. Sabse aasaan tha topic ghumaana, joke maar dena. Tune nahi kiya. 🥺 / Pata hai teen saal main sochti rahi — agar us raat kuch alag hota toh? Aur ab tu yahaan khada hai, mere saamne, poori tarah real. / Aaj raat kisi ko mat batana. Ye wala tu… ye sirf mere liye tha. Good night. ✨</t>
+        </is>
+      </c>
       <c r="O6" s="2" t="inlineStr"/>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="P6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr">
         <is>
           <t>House Watch: terrace pe raat 1 baje 2 log, no cameras rolling, sirf coffee. hum kuch nahi keh rahe par… hum sab dekh rahe hain 👀 #CreatorHouse</t>
         </is>
@@ -907,12 +925,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Cool ban — aage badh ja</t>
+          <t>Bolo ki ab kyun aa rahe ho — 3 saal pehle kahaan thi?</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Halke mein le, deep mat ja. Guard upar, banda safe. (crush -2, fame +1)</t>
+          <t>Sach, par pehle hisaab. Teen saal ka sawaal seedha rakh de. (crush −2, fame +1)</t>
         </is>
       </c>
       <c r="J7" s="2" t="n">
@@ -923,21 +941,22 @@
           <t>ananya −2</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>{crush} → Haha okay, points for the comeback. 😅 / Maine socha shayad… chhodo. Camera off tha, socha asli waala milega. Mera hi vehem tha shayad. / Anyway good night. Kal phir se sab apne masks pehen lenge — tere paas toh already ready hai. 🙂</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>ananya → Seedha vaar. 😅 …theek hai. Is sawaal ka haq banta hai tera. / 3 saal pehle main dar gayi thi. Tune kabhi bola nahi, maine kabhi poocha nahi — aur waqt haath se nikal gaya. / Ab kyun? …pata nahi. Par tu poochta raha, matlab kuch abhi bhi bacha hai. Bas… aaj raat nahi. Good night. 🙂</t>
+        </is>
+      </c>
       <c r="O7" s="2" t="inlineStr"/>
-      <c r="P7" s="2" t="inlineStr">
-        <is>
-          <t>House Watch: koi terrace pe gaya, coffee li, aur 5 min mein wapas neeche. cold. ya bas thaka hua? raat abhi jawaan hai 🌙</t>
+      <c r="P7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>House Watch: 1 baje terrace pe do log — coffee se shuru, phir kuch purana ubhar aaya. dono ke chehre badle hue wapas aaye. halka nahi tha ye 👀🌙 #CreatorHouse</t>
         </is>
       </c>
     </row>
@@ -962,9 +981,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Sab so gaye hain. Kitchen ki ek light jal rahi hai aur Zoya wahin khadi hai — do chai ke mug, ek tumhare liye. "Baitho na. Camera bhi so gaya ab."
-Woh sweet hai, bahut sweet. "Main tumhe pasand karti hoon, sach mein. Isliye keh rahi hoon — is ghar mein har koi tumhare peeche kuch na kuch bol raha hai. Mujhe sab pata chalta hai. Main tumhe bata sakti hoon… agar hum ek-doosre ke saath hon."
-Phir woh halka sa jhukti hai: "Waise… Ria ke baare mein tumhe kya laga? Sach-sach. Yeh baat bas hum dono ke beech rahegi." Uski aankhein muskura rahi hain, par sun woh ek naam ke liye rahi hai.</t>
+          <t>1 AM. Poora ghar so chuka hai. Kitchen ki ek akeli light — aur Zoya, do mug chai ke saath, jaise tumhaara hi intezaar kar rahi ho.
+Zoya: Baitho na babe. Camera bhi so gaya. Main sirf ye dekhna chahti thi tum theek ho ya nahi. 🫶
+Woh chai aage badhaati hai. Meethi awaaz, warm smile. "Is ghar mein sab tumhaare peeche kuch na kuch bol rahe hain. Mujhe sab pata chalta hai. Chaho toh main tumhe intel de sakti hoon."
+Zoya: Bas ek cheez — Ria ke baare mein tumhe sach mein kya lagta hai? Ye baat sirf hum dono ke beech. 👀
+Uski aankhein hass rahi hain. Par tumhe pata hai — Zoya ki har baat ka ek screenshot hota hai. Jo aaj tum bologe, kal woh kisi aur ke phone mein ho sakta hai.
+Zoya: Aur babe… ek aakhri baat. 🤫 Kal raat, terrace, 1 baje — tum aur Ananya, coffee. Maine dekha. Kisi ko bataya nahi… abhi tak.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -984,7 +1006,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Uska trust jeeto. Par ab tum uske karzdaar ho.</t>
+          <t>Uska trust jeeto. Par ab tum uske karzdaar ho — aur woh terrace waali baat uske paas hai. (fame +2, zoya +3)</t>
         </is>
       </c>
       <c r="J8" s="2" t="n">
@@ -995,19 +1017,20 @@
           <t>zoya +3</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>zoya → Uff, mujhe pata tha tum smart ho. 🫶 / Ria ke bare mein jo tumne bola na… honestly same. Hum dono ki wavelength match karti hai babe. / Ab tum meri team ho. Jo bhi ghar mein hota hai, sabse pehle tumhe pata chalega. Bas ek din main bhi tumse ek chhoti si help maangungi. 💅</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>zoya → Uff, mujhe pata tha tum smart ho. 🫶 / Ria ke bare mein jo tumne bola na… honestly same. Hum dono ki wavelength match karti hai babe. / Aur woh terrace waali baat? 🤫 Hamare beech. Main tumhaari side hoon ab. Bas ek din main bhi tumse ek chhoti si help maangungi. 💅</t>
+        </is>
+      </c>
       <c r="O8" s="2" t="inlineStr"/>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="P8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr">
         <is>
           <t>zoya: 1 AM kitchen talks with my new fav in the house 🫶 sabse pyaari energy yahin hai! #CreatorHouse #Day2</t>
         </is>
@@ -1046,7 +1069,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Safe raho. Zoya ko yeh pasand nahi aayega.</t>
+          <t>Safe raho. Par Zoya ke paas ab woh terrace waala patta hai — aur woh khush nahi. (fame −1, zoya −2)</t>
         </is>
       </c>
       <c r="J9" s="2" t="n">
@@ -1057,19 +1080,20 @@
           <t>zoya −2</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>zoya → Aww, koi baat nahi. 🫶 / Tum thoda guarded ho, cute hai. Main bura nahi maan rahi, promise. / Bas ek chhoti si baat babe — jo log meri chai nahi peete na, unke baare mein log baaki cheezein bahut jaldi maan lete hain. Sochna. ✨</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>zoya → Aww, koi baat nahi. 🫶 / Tum thoda guarded ho, cute hai. Main bura nahi maan rahi, promise. / Bas ek baat babe — jinke terrace pe 1 baje "coffee dates" hote hain 👀, unke secrets zyada der secret nahi rehte. Sochna. ✨</t>
+        </is>
+      </c>
       <c r="O9" s="2" t="inlineStr"/>
-      <c r="P9" s="2" t="inlineStr">
+      <c r="P9" s="2" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr">
         <is>
           <t>House Watch: zoya ne midnight chai offer ki aur reply mila poker face 🧊 babe ne dushman bana liya day 2 pe?? 🍿 #CreatorHouse</t>
         </is>
@@ -1096,9 +1120,10 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Dopahar. Sab ke saamne, camera on. Ria tumhaare paas aati hai — perfectly lit, perfectly calm. "Main soch rahi thi hum ek collab karein. Mera reach tumhaare content ko ek hi din mein double kar dega."
-Woh muskura ke ek line jodti hai: "Bas ek chhoti si baat — caption aur credit main handle karungi. Aur agli baar jab main kisi cheez pe stand loon, tum mere saath khadi rahogi. Fair hai na?"
-Poora ghar dekh raha hai. Yeh reach ek tohfa hai — par Ria kabhi muft mein kuch nahi deti. Haan bolo, toh tum uske under aa jaate ho. Naa bolo, toh camera pe tumne queen bee ko reject kiya.</t>
+          <t>Dopahar. Camera roll ho raha hai, poora ghar hall mein hai. Ria seedhi tumhaare saamne aa khadi hoti hai — bilkul composed, jaise scene usne pehle likha ho.
+Ria: Ek collab karte hain. Mera reach tumhaare numbers ek din mein double kar dega. Simple maths hai. 👑
+Ria: Caption aur credit main dekh lungi. Aur jab main kisi cheez pe stand loon, tum mere saath. Bas itna. Fair hai na?
+Reach asli hai — ek collab aur tumhaari follower line upar chali jayegi. Par yeh Ria ka ghar hai, aur uska tohfa hamesha ek zanjeer ke saath aata hai.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1118,7 +1143,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Follower jump pakka. Par ab tum Ria ke karze mein ho.</t>
+          <t>Follower jump pakka. Par ab tum Ria ke karze mein ho. (fame +4, ria +2)</t>
         </is>
       </c>
       <c r="J10" s="2" t="n">
@@ -1129,25 +1154,26 @@
           <t>ria +2</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>Post</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr"/>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr">
         <is>
           <t>Collab drop 🚨 @riaofficial ke saath. Reach dekh ke khud shocked hoon 📈👑 #CreatorHouse #Day2</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
+      <c r="P10" s="2" t="inlineStr">
         <is>
           <t>ria: Good choice. You understand how this house works. Welcome to the top table. 👑
 zoya: Oho, itni jaldi Ria ki team? 💅 noted babe.
-creator.tea: day 2 aur already queen ki chhatri ke neeche 🌂 smart ya scared? 👀</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr">
+Creator Tea: day 2 aur already queen ki chhatri ke neeche 🌂 smart ya scared? 👀</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
         <is>
           <t>House Watch: BREAKING: newbie ne Ria ka collab le liya 📈 reach toh milegi par is ghar mein muft kuch nahi milta 👑🔗 #CreatorHouse #Day2</t>
         </is>
@@ -1186,7 +1212,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Apna naam, apni sharton pe. Reach chhoti, respect apni.</t>
+          <t>Apna naam, apni sharton pe. Reach chhoti, respect apni. (fame −1, ria −3)</t>
         </is>
       </c>
       <c r="J11" s="2" t="n">
@@ -1197,19 +1223,20 @@
           <t>ria −3</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>ria → Interesting. Tumne mana kar diya. 👑 / Bahadur ho, ya naye ho — abhi decide nahi kar paayi. / Koi baat nahi. Main offers ek baar karti hoon. Dekhte hain akele apni reach kitni door le jaati hai. 🤍</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr"/>
       <c r="O11" s="2" t="inlineStr"/>
-      <c r="P11" s="2" t="inlineStr">
+      <c r="P11" s="2" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr">
         <is>
           <t>ria: Some people build their own name. Respect. Dekhte hain woh name kitna bada hota hai. 🤍 #CreatorHouse</t>
         </is>
@@ -1236,9 +1263,11 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Eviction ki pehli raat. Andar sab shaant hai, par bahar internet phatt raha hai. Tumhaara naam trend kar raha hai — aur uske aage ek shabd: "EVICTED?"
-Har follower count ab ek vote jaisa lagta hai. Ghar ke andar tumhe apni standing dikhti hai numbers mein — aur abhi woh number hil raha hai. Neend nahi aa rahi. Phone haath mein hai.
-Tumhe ek post daalna hai — apni worth prove karne ke liye. Do raaste hain: ek honest, dil se — ya ek bada viral swing jo ya toh tumhe bacha lega ya doobo dega.</t>
+          <t>2 AM. Eviction ki pehli raat. Ghar ke andar silence, par phone ki screen jal rahi hai — tumhaara naam trend kar raha hai, aur uske saath ek sawaal: kya tum jaa rahe ho?
+Yeh ghar tumhe ek hi cheez se aaina dikhata hai — followers. Har number ek vote hai. Aur abhi, woh number thehra nahi hai. Woh gir sakta hai.
+Kabir: Suno. Sab bahar tere naam pe bakwaas kar rahe hain. Toh unko jawab de — ek post. Aisa jo sirf tu de sakta hai. 🔥
+Do raaste. Ek honest, kaanpta hua sach — dil se. Ek bada viral swing — spectacle, risk, ya toh raat bacha legi ya doobo degi.
+» Yeh post tumhaara audience read hai. Kal subah follower count batayega tum bache ya nahi. Kaise khelte ho?</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1265,25 +1294,26 @@
         <v>2</v>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>Post</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr"/>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
         <is>
           <t>Sach bolun? Aaj raat dar lag raha hai jaane ka. Par main yahan apna asli self le ke aaya hoon — chahe kal rahoon ya na. Agar meri kahaani tumhe touch karti hai, saath raho. 🤍 #CreatorHouse #DangerNight</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="P12" s="2" t="inlineStr">
         <is>
           <t>kabir: Bhai ye mazaak nahi tha, seedha dil mein laga. Sun — tu kahin nahi jaa raha. Numbers gir bhi jaayein, main yahin khada hoon. Aaj so ja, main jaag raha hoon. 🔥
 ananya: Yeh… itna real tha ki main ro padi. 🥺 Please mat jaana.
 housewatch_india: koi strategy nahi, sirf sach 🥺 vote button dhoondh rahi hoon SAVE ke liye #CreatorHouse</t>
         </is>
       </c>
-      <c r="P12" s="2" t="inlineStr">
+      <c r="Q12" s="2" t="inlineStr">
         <is>
           <t>House Watch: danger night pe koi drama nahi, sirf sach 🥺 vote chatter on fire — SAVE trend kar raha hai. follower rank abhi bhi hilta hua 📉📈 #CreatorHouse #Day2</t>
         </is>
@@ -1329,25 +1359,26 @@
         <v>4</v>
       </c>
       <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>Post</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr"/>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr">
         <is>
           <t>Agar aaj meri last night hai is ghar mein… toh main aise nahi jaaunga. 🎬 Watch this. Sound ON. Yeh reel ya toonga viral kar dega ya main history ban jaaunga. Tumhaara ek share = ek vote. LET'S GO 🔥🚀 #CreatorHouse #DangerNight</t>
         </is>
       </c>
-      <c r="O13" s="2" t="inlineStr">
+      <c r="P13" s="2" t="inlineStr">
         <is>
           <t>kabir: AREY YE KYA THA 😭🔥 poora daao laga diya bhai. Sun — chahe chal jaaye ya na, tu kahin nahi jaa raha. Numbers refresh mat karta reh, so ja. Main dekhta hoon. 🔥
 ria: Bold. Ya tum genius ho ya tumne khud ko abhi dubaya. Kal pata chalega. 👑
 creator.tea: ye banda danger night pe SPECTACLE de raha hai?? 🍿 either legend or gone by morning 👀</t>
         </is>
       </c>
-      <c r="P13" s="2" t="inlineStr">
+      <c r="Q13" s="2" t="inlineStr">
         <is>
           <t>House Watch: EVICTION NIGHT SWING 🎬🚀 ya to tonight ka biggest moment ya biggest flop. followers uchhal rahe hain, vote timeline pagal ho gayi 🔥 #CreatorHouse #Day2</t>
         </is>
@@ -1374,9 +1405,11 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Subah. Ananya tumhe corner mein pakad leta hai — phone haath mein, screen pe ek half-edited reel. "Ek idea hai. Hum dono. Ek collab. Tumhaara reach, meri edit, chemistry toh dikh hi rahi hai."
-Numbers ke hisaab se — Ananya ke followers tumse kam hain. Par yeh reel? Yeh explode kar sakta hai. Dono ke liye. Aur ghar ke andar sab dekh lenge ki tum kiske saath khade ho.
-Ananya ki aankhein excited hain, thodi dari hui bhi. "Sirf haan-na chahiye. Zyaada mat socho."</t>
+          <t>Subah. Ananya tumhe ek taraf le jaata hai — phone pe ek reel adhoora ruka hua, cut hone ka intezaar karta.
+Ananya: Hum dono. Ek collab. Tumhaara reach, meri edit… chemistry toh sabko dikh rahi hai na? 🥺
+Ghar mein aisa collab ek statement hota hai. Sab dekh lenge tum kiski team mein ho — aur Ria bhi.
+Ananya: Sirf haan-na chahiye. Numbers pe mat jaao… bas humpe jaao. ✨
+» Ek reel jo dono ko upar le jaaye — par tumhaare gale mein ek target bhi baandh de. Followers ka juaa, ya safe lane?</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1407,25 +1440,26 @@
           <t>ananya +4</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>Post</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr"/>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr">
         <is>
           <t>Naya duo just dropped 🔥 Ananya + main, ek hi frame mein. Baaki log noticing karte raho. 😌✨ #CreatorHouse #CollabSzn</t>
         </is>
       </c>
-      <c r="O14" s="2" t="inlineStr">
+      <c r="P14" s="2" t="inlineStr">
         <is>
           <t>ananya: Tumne haan kaha… numbers dekhe bina. Yeh yaad rahega mujhe. 🥺✨
 ria: Cute little collab. Reach lend karna generous hota hai… hope it's mutual. 👀
 housewatch_india: RUKO YEH DUO?? day 3 aur main already invested 😭 ship ho gaya bhai</t>
         </is>
       </c>
-      <c r="P14" s="2" t="inlineStr">
+      <c r="Q14" s="2" t="inlineStr">
         <is>
           <t>House Watch: collab reel = soft launch confirmed?? 👀 ye duo ghar ka favourite ban gaya raatoraat 🚢💕 #CreatorHouse</t>
         </is>
@@ -1475,19 +1509,20 @@
           <t>ananya −2</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>ananya → Samajh gaya. Abhi timing sahi nahi hai. Theek hai. 🙂 / Pata tha shayad. Yahan sab pehle apna number dekhte hain, phir banda. / Koi baat nahi yaar. Main akele bhi bana leta hoon. Hamesha se banaya hai. 🥺</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>ananya → Samajh gayi. Abhi timing sahi nahi hai. Theek hai. 🙂 / Pata tha shayad. Yahan sab pehle apna number dekhte hain, phir banda. / Koi baat nahi yaar. Main akele bhi bana leti hoon. Hamesha se banaya hai. 🥺</t>
+        </is>
+      </c>
       <c r="O15" s="2" t="inlineStr"/>
-      <c r="P15" s="2" t="inlineStr">
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr">
         <is>
           <t>ria: Smart. Apna lane protect karna maturity hai. Feelings baad mein, followers pehle. Noted. 🤍 #CreatorHouse</t>
         </is>
@@ -1504,204 +1539,211 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
+          <t>D3-NOM</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Nominations</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Ghar ki lights red ho jaati hain. Production: "Is hafte ki nominations." Sab line mein, koi hil nahi raha.
+Dev: (shaant) Jo hona hai ho jaayega. Main apni journey se khush hoon.
+Screen pe do naam ruk jaate hain — Dev aur Kabir. Kabir ki nazar ek pal ke liye tumse takraati hai.
+Kabir: Dekh… main theek hoon. Sach. Tu mere liye apna number mat girana, samjha? Ye meri ladai hai. 🙂
+» Tumhaara sabse apna banda is hafte ja sakta hai. Abhi — reassure karte ho, ya apna game bachate ho?</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Kabir khatre mein hai — abhi kya karte ho?</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Kabir ko bharosa do — "main hoon"</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Emotional commitment. Woh jaanta hai tum saath ho. (ally +3)</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>kabir +3</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>kabir → Bhai… tune abhi jo kaha na. 🥺 Is ghar mein koi aisa nahi bolta. / Chahe main jaun ya rahoon — tu mera banda hai. Par sun, apna number soch samajh ke kharch karna. Main keh raha hoon.</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr"/>
+      <c r="P16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>kabir: is ghar mein ek banda mila jo mere liye khada raha, bina soche 🥺 baaki sab apna number dekh rahe the #CreatorHouse #Nominations</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>D3-NOM</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Nominations</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Cool raho — apna game bachao</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Yahan har koi apni ladta hai. Standing pehle. (ally −2)</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>kabir −2</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>kabir → Haan haan, samajh gaya. Har koi apni ladta hai. 🙂 / Koi baat nahi bhai. Dekhte hain kal raat kaun kiske liye khada hota hai.</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr"/>
+      <c r="P17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>House Watch: nominations aate hi loyalties saaf dikhne lagti hain 👀 kaun kiske liye number kharch karega, kal raat pata chalega 🍿 #CreatorHouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Afternoon</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
           <t>D3-2</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Zoya Ka Hisaab</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Dopahar mein phone garam ho jaata hai. Zoya ne ek story daali hai — bina naam liye, par sab samajh gaye. "Kuch log itni jaldi 'connection' dikhate hain… lagta hai clout ke liye hai, feelings ke liye nahi. Bas keh rahi hoon. 💅"
-Screenshots already ghoom rahe hain. Comments mein tumhaara aur Ananya ka naam ek saath ghisela ja raha hai. Yeh Zoya ka classic move hai — deniable, meethi shakal, chaaku andar.
-Zoya paas se guzarti hai, muskurate hue. "Oh, tujhe bura laga? Maine toh kisi ka naam bhi nahi liya. 💅"</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Dopahar. Phone vibrate karta hai. Zoya ki ek 'no-name' story — par ghar ka har banda jaanta hai kiski baat ho rahi hai.
+Zoya: Kuch log 'connection' clout ke liye dikhate hain, feelings ke liye nahi. Bas keh rahi hoon. Naam thodi liya maine. 💅
+Screenshots ghoom rahe hain. Comments mein tumhaara aur Ananya ka naam saath mein ghisa ja raha hai.
+Zoya: Oh, chubh gaya? Maine toh naam bhi nahi liya babe. Jise lage uski baat hai. ✨👀
+» Heat lag chuki hai — aur camera ke saamne. Ise blast karke viral karo, ya andar-andar bujha do?</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Zoya ki leak ka kya karte ho?</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Saamne se clap back karo</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>Public jawab. Loud, sharp, viral.</t>
         </is>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="J18" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>zoya −1</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>Post</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr">
         <is>
           <t>Jinki apni koi story nahi hoti, woh dusron ki banate hain. Meri 'clout' meri mehnat hai, kisi ke screenshot se nahi. Namaste. 🙏🔥 #CreatorHouse</t>
         </is>
       </c>
-      <c r="O16" s="2" t="inlineStr">
+      <c r="P18" s="2" t="inlineStr">
         <is>
           <t>zoya: Ooh, itna react? Chhoti si baat pe itna gussa… interesting babe. 💅👀
 ria: Clapping back gives it oxygen, darling. But the delivery… okay, that landed. 👀
 housewatch_india: NAMASTE ke saath bola?? 😭🔥 zoya ko public mein rakh diya, ye clip viral pakka</t>
         </is>
       </c>
-      <c r="P16" s="2" t="inlineStr">
+      <c r="Q18" s="2" t="inlineStr">
         <is>
           <t>House Watch: ZOYA ne story daali, unhone NAMASTE ke saath jawaab diya 😭🔥 ye beef officially on hai #CreatorHouse</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Afternoon</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>D3-2</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Zoya Ka Hisaab</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr"/>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>Chup se control karo</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>Kabir ke saath quiet mein defuse karo.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>kabir +2, zoya −1</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>kabir → Bhai react mat kar, wahi toh chahti hai woh. 😭 Silence se jyada kuch nahi jalta uske liye. / Screenshots ka scene main dekh leta hoon — kaun forward kar raha hai, pata laga leta hoon. / Tu bas normal reh. Do din mein log bhool jaayenge. Main hoon na peeche. 🔥</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr"/>
-      <c r="O17" s="2" t="inlineStr"/>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>ria: No reaction? Interesting. Silence bhi ek strategy hai… ya darr. Time batayega. 🤍 #CreatorHouse</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Late Night</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>D3-3</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Do Dil, Do Raaste</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Raat. Sab so gaye hain. Ananya chhat pe milta hai tumhe — Zoya wale drama ke baad thoda toota hua, thoda himmat karke. "Din bhar sochta raha. Ye jo humaare beech hai… mujhe iska pata karna hai. Sach mein."
-"Par mujhe pata hai tumhaara standing abhi hilaa hua hai. Agar hum aur kareeb aaye, toh log aur baatein banayenge. Tumhaare followers ko farak padega." Ananya ruk jaata hai. "Toh main bas ye jaanna chahta hoon — main pehle aata hoon, ya game?"
-Koi camera nahi. Koi caption nahi. Sirf tum, Ananya, aur ek sawaal jo tum tal nahi sakte.</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Ananya ki baat ka kya jawab dete ho?</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Ananya ko chuno</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>Game ruk sakta hai. Ye feeling nahi.</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>ananya +6</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>ananya → Tum… tumne mujhe chuna. Followers se pehle. 🥺 / Pata hai game mein ye mehenga pad sakta hai. Par tumne phir bhi kaha. Yahi sabse zyaada matter karta hai. / Main tumhaare saath hoon. Ab ye 'almost-something' nahi raha… ye kuch hai. ✨</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="inlineStr"/>
-      <c r="O18" s="2" t="inlineStr"/>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>ananya: kuch cheezein followers se zyaada keemti hoti hain. aaj samajh aaya. 🌙✨ #nofilter</t>
         </is>
       </c>
     </row>
@@ -1711,17 +1753,17 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Late Night</t>
+          <t>Afternoon</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>D3-3</t>
+          <t>D3-2</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Do Dil, Do Raaste</t>
+          <t>Zoya Ka Hisaab</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
@@ -1733,43 +1775,44 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Game ko chuno</t>
+          <t>Chup se control karo</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Yahan followers hi survival hai. Abhi nahi.</t>
+          <t>Kabir ke saath quiet mein defuse karo.</t>
         </is>
       </c>
       <c r="J19" s="2" t="n">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>ananya −3</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr">
+          <t>kabir +2, zoya −1</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
-        <is>
-          <t>ananya → Game. Samajh gaya. Tumne saaf keh diya, uske liye shukriya. 🙂 / Main galat nahi thi ki himmat ki… bas timing shayad galat thi. Ya bandaa. / Theek hai. Main peeche hat jaati hoon. Apna game khelo — main dekhungi. 🥺</t>
-        </is>
-      </c>
-      <c r="N19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>kabir → Bhai react mat kar, wahi toh chahti hai woh. 😭 Silence se jyada kuch nahi jalta uske liye. / Screenshots ka scene main dekh leti hoon — kaun forward kar raha hai, pata laga leta hoon. / Tu bas normal reh. Do din mein log bhool jaayenge. Main hoon na peeche. 🔥</t>
+        </is>
+      </c>
       <c r="O19" s="2" t="inlineStr"/>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>House Watch: chhat pe kuch hua raat ko… dono ki body language subah se ajeeb hai 👀 kuch toot gaya kya? #CreatorHouse</t>
+      <c r="P19" s="2" t="inlineStr"/>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>ria: No reaction? Interesting. Silence bhi ek strategy hai… ya darr. Time batayega. 🤍 #CreatorHouse</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
@@ -1778,24 +1821,26 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>D4-1</t>
+          <t>D3-3</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Doosri Danger Raat</t>
+          <t>Do Dil, Do Raaste</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Speaker phir crackle karta hai. Doosri danger raat. Par is baar naam padhne se pehle hi tum jaan jaate ho — kyunki jo neeche hai, woh tum nahi ho.
-Screen pe Kabir ka naam. Sabse kam standing. Aur ghar mein sirf ek banda ke paas itni reach hai ki usse upar kheench sake — tum.
-Tumhare paas apni standing hai. Usse spend kar sakte ho — Kabir ko bacha lo, apne kharche pe. Ya khud ko upar rakho, aur usse girne do.</t>
+          <t>Raat. Chhat khaali hai, sab so gaye. Ananya tumhaara intezaar kar raha tha — Zoya ke drama ke baad thoda toota, thoda himmat jod ke.
+Ananya: Din bhar yahi socha. Jo humaare beech hai… mujhe sach mein iska pata karna hai. 🥺
+Par Ananya ye bhi jaanta hai — tumhaara game abhi kamzor hai. Kareeb aaye toh followers ko chubhega.
+Ananya: Main bas ek cheez jaanna chahta hoon… main pehle aata hoon, ya tumhaara game? ✨
+» Koi camera nahi, koi caption nahi. Sirf tum aur woh sawaal — dil ya followers?</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Kabir khatre mein hai. Apni standing kharch karke bachaoge?</t>
+          <t>Ananya ki baat ka kya jawab dete ho?</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1805,12 +1850,12 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Usse shield karo — apni standing lagaa do</t>
+          <t>Ananya ko chuno</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Apne followers ki keemat pe Kabir ko upar kheencho. Dosti pehle.</t>
+          <t>Game ruk sakta hai. Ye feeling nahi.</t>
         </is>
       </c>
       <c r="J20" s="2" t="n">
@@ -1818,30 +1863,31 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>kabir +5</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
+          <t>ananya +6</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
-        <is>
-          <t>kabir → Bhai tune… poora din mujhpe laga diya. 😭 / Main dekh raha tha tera number gir raha tha aur tu phir bhi mujhe tag karta gaya. Tune apni jagah ka risk liya. Mere liye. Ye ghar mein koi nahi karta. / Main jokes bahut maarta hoon na, isliye log samajhte hain mujhe kuch farak nahi padta. Aaj padta hai. Tu mera banda hai. Ye main marte dum tak yaad rakhunga. 🔥</t>
-        </is>
-      </c>
-      <c r="N20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>ananya → Tum… tumne mujhe chuna. Followers se pehle. 🥺 / Pata hai game mein ye mehenga pad sakta hai. Par tumne phir bhi kaha. Yahi sabse zyaada matter karta hai. / Main tumhaare saath hoon. Ab ye 'almost-something' nahi raha… ye kuch hai. ✨</t>
+        </is>
+      </c>
       <c r="O20" s="2" t="inlineStr"/>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>House Watch: danger night par apna number GIRA ke bestie ko bachaya?? loyalty over followers is CRAZY work 🥹🔥 protect this one #CreatorHouse #DangerNight</t>
+      <c r="P20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>ananya: kuch cheezein followers se zyaada keemti hoti hain. aaj samajh aaya. 🌙✨ #nofilter</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
@@ -1850,12 +1896,12 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>D4-1</t>
+          <t>D3-3</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Doosri Danger Raat</t>
+          <t>Do Dil, Do Raaste</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
@@ -1867,177 +1913,186 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
+          <t>Game ko chuno</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Yahan followers hi survival hai. Abhi nahi.</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>ananya −3</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>ananya → Game. Samajh gayi. Tumne saaf keh diya, uske liye shukriya. 🙂 / Main galat nahi thi ki himmat ki… bas timing shayad galat thi. Ya bandaa. / Theek hai. Main peeche hat jaati hoon. Apna game khelo — main dekhungi. 🥺</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr"/>
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>House Watch: chhat pe kuch hua raat ko… dono ki body language subah se ajeeb hai 👀 kuch toot gaya kya? #CreatorHouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Late Night</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>D4-1</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Doosri Danger Raat</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Raat. Living room. Sab ek line mein khade hain. Speaker on hota hai — doosri danger raat. Aaj kisi ek ka naam sabse neeche hai.
+Screen roshan hota hai. Number sabke saamne. Tumhari nazar naam pe padti hai — aur tumhare seene mein kuch girta hai. Woh Kabir hai.
+Kabir: Aye… ye toh main hoon bhai. 😭 Koi na, hota hai. Tu apna khyaal rakh. Seriously — mere liye risk mat lena, tera number bhi safe nahi hai.
+Aur tabhi tumhe apni power dikhti hai. Tumhari reach itni hai ki agar tum aaj poora din Kabir ko push karo — reels, tags, story — toh woh bach sakta hai. Par tumhari apni standing girega.
+» Bachana hai toh apne kharche pe. Apne followers, uski jaan. Ya khud ko upar rakho, aur usse akele girne do. Kya karoge?</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Kabir khatre mein hai. Apni standing kharch karke bachaoge?</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Usse shield karo — apni standing lagaa do</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Apne followers ki keemat pe Kabir ko upar kheencho. Dosti pehle.</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>-2</v>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>kabir +5</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>savedAlly=1</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>kabir → Bhai tune… poora din mujhpe laga diya. 😭 / Main dekh raha tha tera number gir raha tha aur tu phir bhi mujhe tag karta gaya. Tune apni jagah ka risk liya. Mere liye. Ye ghar mein koi nahi karta. / Main jokes bahut maarta hoon na, isliye log samajhte hain mujhe kuch farak nahi padta. Aaj padta hai. Tu mera banda hai. Ye main marte dum tak yaad rakhunga. 🔥</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr"/>
+      <c r="P22" s="2" t="inlineStr"/>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>House Watch: danger night par apna number GIRA ke bestie ko bachaya?? loyalty over followers is CRAZY work 🥹🔥 protect this one #CreatorHouse #DangerNight</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Late Night</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>D4-1</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Doosri Danger Raat</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
           <t>Khud ko protect karo — usse girne do</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>Apni standing pehle. Danger raat mein sabse pehle khud.</t>
         </is>
       </c>
-      <c r="J21" s="2" t="n">
+      <c r="J23" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>kabir −3</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr">
         <is>
           <t>Post</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr"/>
-      <c r="N21" s="2" t="inlineStr">
+      <c r="N23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr">
         <is>
           <t>Is ghar mein har koi apni ladai khud ladta hai. Main apni lad raha hoon. 🎯 #DangerNight #CreatorHouse</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="P23" s="2" t="inlineStr">
         <is>
           <t>ria: Finally. Someone who understands the game isn't a group project. Cold, but correct. 👑
 zoya: hii babe survival instinct on point 💅 kuch log doobne wale ko bacha ke khud doob jaate hain. tum smart nikle.
 housewatch_india: left the bestie on the danger board to save their OWN number?? cold blooded 😭 #CreatorHouse</t>
         </is>
       </c>
-      <c r="P21" s="2" t="inlineStr">
+      <c r="Q23" s="2" t="inlineStr">
         <is>
           <t>ria: Danger night reveals everyone. Some shield their friends. Some shield their numbers. I respect the honest ones. 👑 #CreatorHouse</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Night</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>D4-2</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>{crush} Ka Faisla</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Danger raat khatam. Ghar so raha hai. Tumhara phone jalta hai — Ananya.
-"Terrace pe hoon. Akeli. Agar tum aana chaaho toh… main yahin hoon." Woh nahi keh raha ki aao. Woh sirf keh raha hai ki darwaza khula hai.
-Jo tumne ab tak chuna hai — usne dekha hai. Ab woh apna faisla tum pe chhod raha hai. Jaaoge?</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Ananya terrace pe hai. Jaoge, ya jaane doge?</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>Terrace pe jaao — usse mil lo</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>Seedhiyaan chadho. Isko aur mat taalo.</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>ananya +5</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="inlineStr">
-        <is>
-          <t>ananya → Tum aa gaye. 🥺 Sach mein aa gaye. / Pata hai, main poori raat khud se keh rahi thi — mat bol isko, kya sochega. Par tum aa gaye, bina maine kuch poore se kahe. Toh shayad main akeli nahi thi jo ye mehsoos kar rahi thi. / Yeh ghar sabko ek performance bana deta hai. Us chhat pe, tumhare saath… main sirf main thi. Bohot arse baad. 3 saal baad, shayad. Thank you. ✨</t>
-        </is>
-      </c>
-      <c r="N22" s="2" t="inlineStr"/>
-      <c r="O22" s="2" t="inlineStr"/>
-      <c r="P22" s="2" t="inlineStr">
-        <is>
-          <t>ananya: Kuch raatein feed pe nahi jaati. Aaj wali unme se ek hai. 🌙✨ #CreatorHouse</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Night</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>D4-2</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>{crush} Ka Faisla</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>Jaane do — phone neeche rakh do</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>Aaj nahi. Sar shaant, dil surakshit.</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>ananya −2</t>
-        </is>
-      </c>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="inlineStr">
-        <is>
-          <t>ananya → Koi baat nahi. So jao. 🙂 / Main thodi der aur baith jaungi yahin. Hawa achhi hai. Tum apna rest lo. / …sach kahun? Ek pal ke liye maine sach mein socha tha ki tum aaoge. Meri galti. Main akele baithne ki aadi hoon waise bhi. Good night. 🥺</t>
-        </is>
-      </c>
-      <c r="N23" s="2" t="inlineStr"/>
-      <c r="O23" s="2" t="inlineStr"/>
-      <c r="P23" s="2" t="inlineStr">
-        <is>
-          <t>ananya: Terrace, akeli, thandi hawa. Itna hi chahiye tha waise bhi. Kisi ka intezaar nahi tha. Bilkul nahi. 🙂🌙 #CreatorHouse</t>
         </is>
       </c>
     </row>
@@ -2052,404 +2107,812 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
+          <t>D4-ELIM</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Eviction</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Production: "Is hafte ghar chhodenge…" — aur screen pe naam jalta hai: Kabir.
+Tumhaara banda. Woh jo har raat tere saath khada tha. Aaj tumne apna number bachaya — aur ye keemat aayi.
+Kabir: Are yaar, ro mat. 😅 Maine bola tha na — har koi apni ladta hai. Tu jeet, mere liye bhi. Bas… yaad rakhna main tere liye khada tha.
+» Darwaaza band. Ghar mein ek Kabir-shaped khaali jagah. Tune game bachaya — par kis keemat par?</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Naam aa gaya. Ise kaise lete ho?</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Kabir ko last hug do</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Guilt aur pyaar. Woh gaya, tu bacha.</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>kabir → (bahar se, voice note) Bhai jeet ke aana. Trophy meri bhi hai 🥺 aur next time apne bande ke liye number gira dena. Love you yaar.</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr"/>
+      <c r="P24" s="2" t="inlineStr"/>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>House Watch: ek aur eviction, ek aur ghar-hilaane waali raat 🥀 kuch bandhan yahin toot jaate hain #CreatorHouse #EvictionNight</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Very Late</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>D4-ELIM</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Eviction</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Chup-chaap dekho jaate hue</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Kuch keh nahi paaye. Sirf dekha.</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>zoya → Dekha? Loyalty se ghar nahi jeeta jaata. Tumne sahi kiya… shayad. 💅</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr"/>
+      <c r="P25" s="2" t="inlineStr"/>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>House Watch: ek aur eviction, ek aur ghar-hilaane waali raat 🥀 kuch bandhan yahin toot jaate hain #CreatorHouse #EvictionNight</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Very Late</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>D4-ELIM</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Eviction  ⑂ shielded ally → Dev out</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Production: "Is hafte ghar chhodenge…" — aur screen pe naam jalta hai: Dev.
+Tumne kal raat apna poora number Kabir pe laga diya tha. Woh bach gaya. Aur Dev — wildcard, hamesha kinaare pe — chala jaata hai.
+Dev: (shaant, ek muskaan) Koi shikaayat nahi. Achhi journey thi. Kabir, apne bande ka khyaal rakhna. 🙏
+Kabir: Bhai… tune sach mein apna number gira ke mujhe bachaya 😭 Main ye zindagi bhar nahi bhoolunga.
+» Dev chala gaya. Kabir bach gaya — tumhaari wajah se. Aaj ka bandhan aur gehra ho gaya.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Naam aa gaya. Ise kaise lete ho?</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Kabir ko gale lagao</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Tumne use bachaya. Ye bond ab pukka.</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>kabir → Bhai jo tune kiya na… main tere liye kuch bhi. Ride or die. Ab finale tak saath 🔥</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr"/>
+      <c r="P26" s="2" t="inlineStr"/>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>House Watch: ek aur eviction, ek aur ghar-hilaane waali raat 🥀 kuch bandhan yahin toot jaate hain #CreatorHouse #EvictionNight</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Very Late</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>D4-ELIM</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Eviction  ⑂ shielded ally → Dev out</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Dev ko respect se vida karo</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Wildcard gaya, sar utha ke.</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>dev → (bahar se) Tune apne dost ke liye jo kiya, woh rare hai. Jeet ke dikhana. Take care. 🙏</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr"/>
+      <c r="P27" s="2" t="inlineStr"/>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t>House Watch: ek aur eviction, ek aur ghar-hilaane waali raat 🥀 kuch bandhan yahin toot jaate hain #CreatorHouse #EvictionNight</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Night</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>D4-2</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>{crush} Ka Faisla</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Danger raat ka shor beh chuka hai. Ghar andhere mein doob gaya hai. Tum jaage ho — dil abhi bhi tez chal raha hai. Phone jalta hai.
+Ananya: So gaye kya? Main terrace pe hoon… akeli. Neeche itna drama tha, upar bas hawa hai aur main. 🥺
+Ananya: Dekho, main tumhe force nahi kar rahi. Bas… agar tum aana chaaho, toh main yahin hoon. Aur agar nahi, toh bhi theek hai. ✨
+Yeh woh Ananya nahi hai jo camera ke saamne guarded rehti hai. Yeh woh hai jisne apna guard neeche rakha hai — sirf tumhare liye. Aur ise pata hai tumne ab tak kya-kya chuna.
+» Woh apna faisla tumhare haath mein de rahi hai. Seedhiyaan chadhoge — ya phone neeche rakh ke so jaaoge? Kya karoge?</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Ananya terrace pe hai. Jaoge, ya jaane doge?</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Terrace pe jaao — usse mil lo</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Seedhiyaan chadho. Isko aur mat taalo.</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>ananya +5</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>ananya → Tum aa gaye. 🥺 Sach mein aa gaye. / Pata hai, main poori raat khud se keh rahi thi — mat bol isko, kya sochega. Par tum aa gaye, bina maine kuch poore se kahe. Toh shayad main akeli nahi thi jo ye mehsoos kar rahi thi. / Yeh ghar sabko ek performance bana deta hai. Us chhat pe, tumhare saath… main sirf main thi. Bohot arse baad. 3 saal baad, shayad. Thank you. ✨</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr"/>
+      <c r="P28" s="2" t="inlineStr"/>
+      <c r="Q28" s="2" t="inlineStr">
+        <is>
+          <t>ananya: Kuch raatein feed pe nahi jaati. Aaj wali unme se ek hai. 🌙✨ #CreatorHouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Night</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>D4-2</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>{crush} Ka Faisla</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Jaane do — phone neeche rakh do</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Aaj nahi. Sar shaant, dil surakshit.</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>ananya −2</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>ananya → Koi baat nahi. So jao. 🙂 / Main thodi der aur baith jaungi yahin. Hawa achhi hai. Tum apna rest lo. / …sach kahun? Ek pal ke liye maine sach mein socha tha ki tum aaoge. Meri galti. Main akele baithne ki aadi hoon waise bhi. Good night. 🥺</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr"/>
+      <c r="P29" s="2" t="inlineStr"/>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>ananya: Terrace, akeli, thandi hawa. Itna hi chahiye tha waise bhi. Kisi ka intezaar nahi tha. Bilkul nahi. 🙂🌙 #CreatorHouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Very Late</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
           <t>D4-3</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Ria, Bina Mask</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>2 AM. Tumhare paas Zoya ke leak kiye screenshots hain — aur unme Ria ka poora sach hai. Woh 2.1M ka glamour udhaar ke paise pe khada hai. Sponsor ka bakaya, brand ki dhamki, sab kuch.
-Ek post. Ek expose. Aur subah tak Ria ki poori image — jo image tumhe din 1 se chhoti mehsoos karati rahi hai — sabke saamne toot jaayegi. Followers tumhare paas aa jaayenge.
-Ya tum ye screenshots delete kar do. Clean raho. Zoya ki gandagi mein haath na daalo. Faisla tumhara.</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>2 AM. Sab so gaye. Tumhare phone pe ek folder — Zoya ne bheja. Screenshots. Aur inme Ria ka woh sach hai jo woh 2 saal se chhupa rahi hai.
+Zoya: hii babe ✨ mila? maine mehnat se nikala ye sab. Ria ki poori 'luxury life' — udhaar ke paise pe. sponsor ke messages, bakaya, sab. 👀
+Zoya: main apne haath ganda nahi karna chahti. par tu? tu post kar de. subah tak woh khatam. aur uske saare followers… idhar. 💅
+Yeh woh Ria hai jisne tumhe din 1 se 'small-town' bola. Jisne tumhe har camera ke saamne chhota mehsoos karaya. Ek tap, aur uska mask utar jaayega.
+» Ek post — Ria khatam, followers tumhare. Ya screenshots delete — clean haath, chhoti reach. Kya karoge?</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Ria ka sach — expose karoge, ya clean rahoge?</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Expose karo — sach post kar do</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>Ria ka mask utaar do. Followers aayenge. Par ye ruthless hai.</t>
         </is>
       </c>
-      <c r="J24" s="2" t="n">
+      <c r="J30" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>ananya −2</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr">
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr">
         <is>
           <t>Post</t>
         </is>
       </c>
-      <c r="M24" s="2" t="inlineStr"/>
-      <c r="N24" s="2" t="inlineStr">
+      <c r="N30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr">
         <is>
           <t>Is ghar mein sabke 'aesthetic' ke peeche kuch aur hota hai. Aaj kuch cheezein sabke saamne rakhta hoon. Truth over image. 👀 #CreatorHouse #Receipts</t>
         </is>
       </c>
-      <c r="O24" s="2" t="inlineStr">
+      <c r="P30" s="2" t="inlineStr">
         <is>
           <t>ria: So this is who you are. Fine. You want my throne? You'll learn how heavy it is. This isn't over. 👑
 zoya: AND SCENE 💅✨ dekha babe? maine kaha tha. tune woh kiya jo mujhe karna tha — aur ilzaam tere sar. genius. 👀
 housewatch_india: NOT THE RECEIPTS 😭😭 ria's whole empire on borrowed money?? this house just went NUCLEAR #CreatorHouse #Exposed</t>
         </is>
       </c>
-      <c r="P24" s="2" t="inlineStr">
+      <c r="Q30" s="2" t="inlineStr">
         <is>
           <t>House Watch: the house is at WAR 🍿 team-exposed vs team-ria… iske baad koi normal nahi reh sakta. dropping everything to watch this 👀🔥 #CreatorHouse #Receipts</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
+    <row r="31">
+      <c r="A31" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>Very Late</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>D4-3</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Ria, Bina Mask</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr"/>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>Clean raho — screenshots delete karo</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>Zoya ke khel mein haath mat daalo. Reach kam, dignity poori.</t>
         </is>
       </c>
-      <c r="J25" s="2" t="n">
+      <c r="J31" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="K25" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>kabir +3</t>
         </is>
       </c>
-      <c r="L25" s="2" t="inlineStr">
+      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
       </c>
-      <c r="M25" s="2" t="inlineStr">
+      <c r="N31" s="2" t="inlineStr">
         <is>
           <t>kabir → Bhai maine dekha Zoya kya bhej rahi thi. Poora ghar us folder ka wait kar raha tha. 😳 / Aur tune delete kar diya. Ria ne tere saath kabhi seedha nahi kiya — tere haath mein usse barbaad karne ka mauka tha, aur tune nahi liya. / Followers baad mein bhi aa jaayenge yaar. Par jo tu aaj raat tha — woh Zoya kabhi nahi ban sakti. Main tujhe iske liye respect karta hoon. Sach. 🔥</t>
         </is>
       </c>
-      <c r="N25" s="2" t="inlineStr"/>
-      <c r="O25" s="2" t="inlineStr"/>
-      <c r="P25" s="2" t="inlineStr">
+      <c r="O31" s="2" t="inlineStr"/>
+      <c r="P31" s="2" t="inlineStr"/>
+      <c r="Q31" s="2" t="inlineStr">
         <is>
           <t>ria: Someone had my life in their hands last night. They chose to walk away clean. I don't forget things like that. Neither the kindness, nor the fact that they could. 🤍 #CreatorHouse</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
+    <row r="32">
+      <c r="A32" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Late Night</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>D5-1</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Aakhri Bada Faisla</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Finale kal hai. Aaj raat house ka aakhri content window khula hai — ek post, prime slot, poora internet dekh raha hai. Ye tumhare number pe seedha asar daalega.
-Ek taraf: ek clean 'winner' move — tumhe, akela, top pe. Fame ke liye perfect. Par isme Ananya ke saath jo build hua, use side pe rakhna padega. Publicly.
-Doosri taraf: ye raat kisi ke saath sach mein bitao — number chhodo, Ananya ko choose karo. Camera ke bina.</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Late night. Villa chup hai. Finale ko chaubees ghante bhi nahi bache. House ka aakhri content window abhi khula hai — ek slot, prime time, saara internet online.
+Ek clean winner move ready hai — sirf tum, top pe, spotlight full. Numbers isse pyaar karenge. Bas Ananya ko frame ke bahar rakhna padega. Sab ke saamne.
+Ananya: Kal sab khatam ho jaayega na? Bas… aaj raat ke liye camera band. Sirf tum aur main. Ho sakta hai? 🥺
+Ek taraf pachaas hazaar log. Doosri taraf ek insaan jo pehli baar sach mein ruka hai.
+» Ye wahi sawaal hai jo Day 1 se chhupa tha — followers, ya feeling? Aaj raat jhooth nahi chalega.</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Aakhri raat — play to win, ya play for the romance?</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>Play to WIN</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>Winner move post karo. Spotlight sirf tumhara.</t>
         </is>
       </c>
-      <c r="J26" s="2" t="n">
+      <c r="J32" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>ananya −4</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="L32" s="2" t="inlineStr"/>
+      <c r="M32" s="2" t="inlineStr">
         <is>
           <t>Post</t>
         </is>
       </c>
-      <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="inlineStr">
+      <c r="N32" s="2" t="inlineStr"/>
+      <c r="O32" s="2" t="inlineStr">
         <is>
           <t>Das din. Ek ghar. Aur main abhi bhi khada hoon — akela, apne dum pe. Kal finale. Baaki sab noise hai. 🏆 #CreatorHouse #FinaleEve</t>
         </is>
       </c>
-      <c r="O26" s="2" t="inlineStr">
+      <c r="P32" s="2" t="inlineStr">
         <is>
           <t>ria: Finale se ek raat pehle solo flex. Cold. Smart. Yahi to game hai. 👑
-ananya: Frame me jagah nahi thi na meri. Samajh gaya. Koi baat nahi. 🙂
+ananya: Frame me jagah nahi thi na meri. Samajh gayi. Koi baat nahi. 🙂
 HouseWatch India: FINALE EVE aur ye banda solo chala gaya 👀 numbers ke liye sab chhod diya. iconic ya ice-cold? #CreatorHouse</t>
         </is>
       </c>
-      <c r="P26" s="2" t="inlineStr">
+      <c r="Q32" s="2" t="inlineStr">
         <is>
           <t>HouseWatch India: Finale eve aur koi prime slot me akela chamak raha hai — apne closest bond ko frame se bahar rakhke. Numbers up. Dil ka pata nahi. 👀🏆 #CreatorHouse #Day5</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="n">
+    <row r="33">
+      <c r="A33" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>Late Night</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>D5-1</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Aakhri Bada Faisla</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>Play for the ROMANCE</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>Slot chhodo. Aaj raat Ananya ke saath, camera ke bina.</t>
         </is>
       </c>
-      <c r="J27" s="2" t="n">
+      <c r="J33" s="2" t="n">
         <v>-4</v>
       </c>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>ananya +6</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
       </c>
-      <c r="M27" s="2" t="inlineStr">
+      <c r="N33" s="2" t="inlineStr">
         <is>
           <t>ananya → Ruko… tumne prime slot chhod diya? Finale se ek raat pehle? 🥺 / Numbers ke liye nahi… mere liye? Sach me? / Chalo terrace pe. Camera band. Aaj raat sirf hum do. Ye… ye maine kabhi kisi ke saath feel nahi kiya. 🌙</t>
         </is>
       </c>
-      <c r="N27" s="2" t="inlineStr"/>
-      <c r="O27" s="2" t="inlineStr"/>
-      <c r="P27" s="2" t="inlineStr">
+      <c r="O33" s="2" t="inlineStr"/>
+      <c r="P33" s="2" t="inlineStr"/>
+      <c r="Q33" s="2" t="inlineStr">
         <is>
           <t>ananya: Kisi ne aaj raat pachaas hazaar log chhod diye… ek insaan ke liye. Main. 🌙 Kal jo bhi ho, ye raat meri hai. #FinaleEve</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="n">
+    <row r="34">
+      <c r="A34" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Finale</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>D5-2</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Live Finale</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>Studio lights. 1.1 lakh log live. Ria, Kabir, Ananya — sab stage pe, sab tumhare saath. Host lifafa kholti hai.
-"Aur is season ka result…" — pause. Poora India saans roke baitha hai.
-Naam tumhara hai. Ye das din is ek pal mein simat gaye. Ab bas — tum ise kaise lete ho?</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Live finale. Studio lights, 1.1 lakh log online. Stage pe Ria, Kabir, Ananya — sab bach gaye, sab tumhare saath khade hain.
+Host: Aur is season ka winner… hai… ye naam. Congratulations. Stage tumhara hai. 🎤
+Taaliyan. Camera tumhare chehre pe zoom hota hai. Kabir ki aankhein bhar aayi. Ananya bas dekh raha hai — jaise sab kuch is ek pal ka tha.
+» Das din. Ek mic. Ab jo bologe — wahi log yaad rakhenge. Ye tumhara hai. Kaise lete ho?</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Result aa gaya — ise kaise lete ho?</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>Own it</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>Ye tumne kamaaya. Poora malik banke lo.</t>
         </is>
       </c>
-      <c r="J28" s="2" t="n">
+      <c r="J34" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K28" s="2" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>ananya +1, kabir +1</t>
         </is>
       </c>
-      <c r="L28" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
       </c>
-      <c r="M28" s="2" t="inlineStr">
+      <c r="N34" s="2" t="inlineStr">
         <is>
           <t>kabir → OYE WINNER 😭🔥 stage pe aise khada tha jaise ghar tera hi tha. mereko pata tha bhai. / haq se liya tune. koi begging nahi. that's my banda. 🔥 / Tumne ise apna banake liya. 🥺 Aur mujhe khushi hai maine tumhe uss raat dekha tha — before everyone else.</t>
         </is>
       </c>
-      <c r="N28" s="2" t="inlineStr"/>
-      <c r="O28" s="2" t="inlineStr"/>
-      <c r="P28" s="2" t="inlineStr">
+      <c r="O34" s="2" t="inlineStr"/>
+      <c r="P34" s="2" t="inlineStr"/>
+      <c r="Q34" s="2" t="inlineStr">
         <is>
           <t>HouseWatch India: AUR WINNER HAI… 🏆 stage pe aisa control jaise trophy pehle se hi inki thi. no shaking, no begging. season over. main character confirmed. 👑 #CreatorHouse #Finale</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="n">
+    <row r="35">
+      <c r="A35" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>Finale</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>D5-2</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>Live Finale</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr"/>
-      <c r="F29" s="2" t="inlineStr"/>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>Grateful / humble</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>Ye akele ka nahi tha. Sab ko lekar lo.</t>
         </is>
       </c>
-      <c r="J29" s="2" t="n">
+      <c r="J35" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>ananya +2, kabir +2</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr"/>
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
       </c>
-      <c r="M29" s="2" t="inlineStr">
+      <c r="N35" s="2" t="inlineStr">
         <is>
           <t>kabir → bhai stage pe humaara naam liya tune 😭 sabke saamne. main ro diya lowkey. / trophy teri, par tune usko sabki bana diya. that's why tu jeeta. 🔥 / Tumne mujhe apne moment me kheencha. 🥺 Winner ho tum — par insaan pehle. Yahi yaad rahega mujhe.</t>
         </is>
       </c>
-      <c r="N29" s="2" t="inlineStr"/>
-      <c r="O29" s="2" t="inlineStr"/>
-      <c r="P29" s="2" t="inlineStr">
+      <c r="O35" s="2" t="inlineStr"/>
+      <c r="P35" s="2" t="inlineStr"/>
+      <c r="Q35" s="2" t="inlineStr">
         <is>
           <t>kabir: mera banda jeet gaya 😭🔥 aur trophy uthake sabse pehle humaara naam liya. yahi banda tha jo jeetne ke laayak tha. #Finale #CreatorHouse</t>
         </is>
@@ -2469,13 +2932,13 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Character</t>
@@ -2488,7 +2951,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Role in the house</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -2510,12 +2973,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>The FOLLOWERS rival — queen bee, huge following, image on borrowed money; poaches, undermines, competes for #1</t>
+          <t>Followers rival — queen bee, image on borrowed money</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Controlled, cutting; compliments that land like warnings</t>
+          <t>controlled, cutting</t>
         </is>
       </c>
     </row>
@@ -2532,12 +2995,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>The HEAT engine — sweet on camera, savage off; leaks, screenshots, deniable drama that threatens your standing</t>
+          <t>Heat engine — sweet on camera, leaks &amp; screenshots off it</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>"hii babe" sweet on surface, sharp in private</t>
+          <t>deniable-sweet</t>
         </is>
       </c>
     </row>
@@ -2554,12 +3017,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>The CRUSH (male player) / ALLY (female player) — an unspoken almost-something from 3 years ago; the romance dial</t>
+          <t>CRUSH (♂ player) / ALLY (♀) — the 3-years-ago almost-something</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Warm, earnest, guarded 🥺✨</t>
+          <t>warm, guarded 🥺</t>
         </is>
       </c>
     </row>
@@ -2576,19 +3039,19 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>The ALLY (male player) / CRUSH (female player) — your ride-or-die whose loyalty gets tested</t>
+          <t>ALLY (♂ player) / CRUSH (♀) — ride-or-die</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Loud, loyal, street-Mumbai funny; soft only with you</t>
+          <t>loud, loyal</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>— Dev —</t>
+          <t>Dev</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -2598,12 +3061,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>CUT in v4 (was the quiet observer). Only 4 NPCs now.</t>
+          <t>Wild-card housemate — the sacrificial nominee (evicted after D4-1)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>understated</t>
         </is>
       </c>
     </row>
@@ -2618,16 +3081,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Ending</t>
@@ -2640,12 +3103,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Title shown</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>What it means</t>
+          <t>Meaning</t>
         </is>
       </c>
     </row>
@@ -2657,7 +3120,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Followers/Fame ≥ 45  AND  Crush bond ≥ 55</t>
+          <t>Fame ≥45 AND Crush ≥55</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2667,7 +3130,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Topped the house AND the romance held. Perfect finale.</t>
+          <t>Won the house + the romance</t>
         </is>
       </c>
     </row>
@@ -2679,7 +3142,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Fame ≥ 45,  bond &lt; 55</t>
+          <t>Fame ≥45, Crush &lt;55</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2689,7 +3152,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Won #1, played everyone — leave alone.</t>
+          <t>Won #1, alone</t>
         </is>
       </c>
     </row>
@@ -2701,7 +3164,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Fame &lt; 45,  bond ≥ 55</t>
+          <t>Fame &lt;45, Crush ≥55</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2711,7 +3174,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Not #1, but walked out with something real.</t>
+          <t>Real romance, lower rank</t>
         </is>
       </c>
     </row>
@@ -2723,7 +3186,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Fame &lt; 45  AND  bond &lt; 55</t>
+          <t>both low</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2733,29 +3196,9 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>The house used you and spat you out.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>NOTE</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Two dials only: FOLLOWERS (deltas.fame — your standing, moved by POSTS) and CRUSH BOND (relationshipDeltas on the crush). The romance compounds D1-3 → D3-3 → D4-2 → D5-1. Resolved in code (resolveEnding).</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
+          <t>Used and dropped</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2768,16 +3211,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="112" customWidth="1" min="1" max="1"/>
+    <col width="104" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
+    <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Creator House — v4 REWRITE (drafted, NOT yet live)</t>
+          <t>Creator House v4 — DRAFT being wired live</t>
         </is>
       </c>
     </row>
@@ -2787,79 +3230,45 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>14 beats across 5 chapters. Cast: Ria, Zoya, Ananya, Kabir (Dev cut).</t>
+          <t>16 beats. Source: public/content/creator-house-v4.json (version 8).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>The app still ships the 29-beat v3 story. This v4 is authored but not integrated/verified yet.</t>
+          <t>⑂ = a branch VARIANT. D4-1 "shield the ally" sets the savedAlly flag; D4-ELIM then branches:</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   shielded → Dev evicted (⑂ row).   not shielded → the ALLY evicted (base row).</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Two goals drive everything:</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>• FOLLOWERS (Fame) — survival / audience standing; moved mainly by your POSTS (~6 post-choices).</t>
+          <t>Tokens resolved for a MALE player: {crush}=Ananya, {ally}=Kabir; gendered verbs → male form.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>• CRUSH BOND — the romance; compounds through the crush beats to the ending.</t>
+          <t>(Female player: crush=Kabir, ally=Ananya, verbs flip.)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Danger nights (D2-3, D4-1) frame your follower standing as survival — dread, never a real game-over.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>How to read Story: each beat has 2 choices (rows); Scene/Q show once (A row).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Every choice does ONE thing — POST (fame moves + house reacts) or a character DM (bond moves).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Tokens resolved for readability (game swaps by gender at runtime):</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   {name}→You  ·  {crush}→Ananya  ·  {ally}→Kabir   (FEMALE player: crush=Kabir, ally=Ananya)</t>
+          <t>Screenshot images in D3-2 (crush-vote) + D4-3 (Ria dirt) are placeholders — to be generated.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ch-v4: publish + flip the loader — Creator House now runs the v4 story
- content.ts bundled import + manifest → creator-house-v4.json (version 9, forces
  any stale v3 cache to supersede). v3 file kept for history.
- Placeholder images for the two screenshot beats (D3-2 crush-vote, D4-3 Ria dirt)
  — real files (no 404); to be replaced with generated screenshots.
- Verified end-to-end: no unresolved gender tokens (♂/♀), and both eviction paths
  resolve (shield→Dev out; don't→ally out, with the D4-3/D5-2 ally-gone cascade).
- Refreshed the v4 story sheet to match live. tsc + 77 tests green.

Players now get the 16-beat Followers+Romance story with the branching eviction.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/creator-house-v4-story.xlsx
+++ b/docs/creator-house-v4-story.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q35"/>
+  <dimension ref="A1:Q39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1368,7 +1368,7 @@
       <c r="N13" s="2" t="inlineStr"/>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Agar aaj meri last night hai is ghar mein… toh main aise nahi jaaunga. 🎬 Watch this. Sound ON. Yeh reel ya toonga viral kar dega ya main history ban jaaunga. Tumhaara ek share = ek vote. LET'S GO 🔥🚀 #CreatorHouse #DangerNight</t>
+          <t>Agar aaj meri last night hai is ghar mein… toh main aise nahi jaaunga. 🎬 Watch this. Sound ON. Yeh reel ya toh viral kar degi ya main history ban jaaunga. Tumhaara ek share = ek vote. LET'S GO 🔥🚀 #CreatorHouse #DangerNight</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1405,7 +1405,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Subah. Ananya tumhe ek taraf le jaata hai — phone pe ek reel adhoora ruka hua, cut hone ka intezaar karta.
+          <t>Subah. Ananya tumhe ek taraf le jaati hai — phone pe ek reel adhoora ruka hua, cut hone ka intezaar karta.
 Ananya: Hum dono. Ek collab. Tumhaara reach, meri edit… chemistry toh sabko dikh rahi hai na? 🥺
 Ghar mein aisa collab ek statement hota hai. Sab dekh lenge tum kiski team mein ho — aur Ria bhi.
 Ananya: Sirf haan-na chahiye. Numbers pe mat jaao… bas humpe jaao. ✨
@@ -1687,11 +1687,11 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Dopahar. Phone vibrate karta hai. Zoya ki ek 'no-name' story — par ghar ka har banda jaanta hai kiski baat ho rahi hai.
-Zoya: Kuch log 'connection' clout ke liye dikhate hain, feelings ke liye nahi. Bas keh rahi hoon. Naam thodi liya maine. 💅
-Screenshots ghoom rahe hain. Comments mein tumhaara aur Ananya ka naam saath mein ghisa ja raha hai.
-Zoya: Oh, chubh gaya? Maine toh naam bhi nahi liya babe. Jise lage uski baat hai. ✨👀
-» Heat lag chuki hai — aur camera ke saamne. Ise blast karke viral karo, ya andar-andar bujha do?</t>
+          <t>Dopahar. Zoya ka ek "no-name" post — par ghar ka har banda jaanta hai kiski baat hai. Neeche comments mein tumhaara aur Ananya ka naam ghisa ja raha hai.
+Screenshot mein Ananya ke apne shabd — kisi aur ko: "usse close rakhna hai, numbers double ho rahe hain." Tumhaari saans ruk jaati hai.
+Zoya: Oh no, chubh gaya? 🙈 Maine toh sirf sach dikhaya babe. Ab pata chala na — is ghar mein "feelings" bhi ek game hoti hain. 👀
+Heat lag chuki hai, aur camera ke saamne. Tumhaara game bhi daao pe, aur dil bhi. Zoya muskura rahi hai — ek teer, do nishaane.
+» Sabke saamne tumhe used dikhaya gaya. Ise blast karke apna sach rakho — ya andar-andar sambhaalo?</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Public jawab. Loud, sharp, viral.</t>
+          <t>Public. Apni izzat khud rakho, chahe drama ho. (fame +3, zoya −1)</t>
         </is>
       </c>
       <c r="J18" s="2" t="n">
@@ -1731,19 +1731,19 @@
       <c r="N18" s="2" t="inlineStr"/>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>Jinki apni koi story nahi hoti, woh dusron ki banate hain. Meri 'clout' meri mehnat hai, kisi ke screenshot se nahi. Namaste. 🙏🔥 #CreatorHouse</t>
+          <t>Screenshots bina context ke sirf aadha sach hote hain. 🎬 Jise strategy samajh rahe ho, woh meri kahaani hai — aur main use kisi ke edit se define nahi hone dunga. #CreatorHouse</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>zoya: Ooh, itna react? Chhoti si baat pe itna gussa… interesting babe. 💅👀
-ria: Clapping back gives it oxygen, darling. But the delivery… okay, that landed. 👀
-housewatch_india: NAMASTE ke saath bola?? 😭🔥 zoya ko public mein rakh diya, ye clip viral pakka</t>
+          <t>zoya: Ooh, fighting spirit 💅 par screenshots screenshots hote hain babe 👀
+ria: Bold. Par ab poora ghar tumhaari "kahaani" ko differently dekhega. 👑
+House Watch: usne screenshots ka jawaab HEAD ON diya 😭🔥 season ka biggest twist #CreatorHouse</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>House Watch: ZOYA ne story daali, unhone NAMASTE ke saath jawaab diya 😭🔥 ye beef officially on hai #CreatorHouse</t>
+          <t>Creator Tea: ZOYA ne screenshots daale, unhone clap back kiya 🍿 team-used vs team-strategy… ghar do hisso mein baant gaya #CreatorHouse</t>
         </is>
       </c>
     </row>
@@ -1775,12 +1775,12 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Chup se control karo</t>
+          <t>Chup se sambhaalo — Kabir ke paas jaao</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Kabir ke saath quiet mein defuse karo.</t>
+          <t>React mat karo, wahi Zoya chahti hai. Andar process karo. (fame −1, ally +2)</t>
         </is>
       </c>
       <c r="J19" s="2" t="n">
@@ -1799,14 +1799,14 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>kabir → Bhai react mat kar, wahi toh chahti hai woh. 😭 Silence se jyada kuch nahi jalta uske liye. / Screenshots ka scene main dekh leti hoon — kaun forward kar raha hai, pata laga leta hoon. / Tu bas normal reh. Do din mein log bhool jaayenge. Main hoon na peeche. 🔥</t>
+          <t>kabir → Bhai react mat kar, wahi toh chahti hai woh 😭 Silence se zyada kuch nahi jalta uske liye. / Aur woh screenshot… sun. Ho sakta hai shuru mein strategy rahi ho. Par maine Ananya ki aankhein dekhi hain jab woh teri baat karti hai. Woh ab fake nahi. / Zoya ne aag lagayi. Tu paani mat ban, aur aag bhi mat. Bas… Ananya se khud poochh, screen ke bahar.</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>ria: No reaction? Interesting. Silence bhi ek strategy hai… ya darr. Time batayega. 🤍 #CreatorHouse</t>
+          <t>House Watch: screenshots viral, par woh banda? poker face 🧊 andar kuch pak raha hai ya sab sambhaal liya? 👀 #CreatorHouse</t>
         </is>
       </c>
     </row>
@@ -1831,10 +1831,10 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Raat. Chhat khaali hai, sab so gaye. Ananya tumhaara intezaar kar raha tha — Zoya ke drama ke baad thoda toota, thoda himmat jod ke.
+          <t>Raat. Chhat khaali hai, sab so gaye. Ananya tumhaara intezaar kar rahi tha — Zoya ke drama ke baad thoda toota, thoda himmat jod ke.
 Ananya: Din bhar yahi socha. Jo humaare beech hai… mujhe sach mein iska pata karna hai. 🥺
-Par Ananya ye bhi jaanta hai — tumhaara game abhi kamzor hai. Kareeb aaye toh followers ko chubhega.
-Ananya: Main bas ek cheez jaanna chahta hoon… main pehle aata hoon, ya tumhaara game? ✨
+Par Ananya ye bhi jaanti hai — tumhaara game abhi kamzor hai. Kareeb aaye toh followers ko chubhega.
+Ananya: Main bas ek cheez jaanna chahti hoon… main pehle aati hoon, ya tumhaara game? ✨
 » Koi camera nahi, koi caption nahi. Sirf tum aur woh sawaal — dil ya followers?</t>
         </is>
       </c>
@@ -2071,7 +2071,11 @@
           <t>kabir −3</t>
         </is>
       </c>
-      <c r="L23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>allyEvicted=1</t>
+        </is>
+      </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
           <t>Post</t>
@@ -2538,7 +2542,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Ria ka mask utaar do. Followers aayenge. Par ye ruthless hai.</t>
+          <t>Ria ka mask utaar do. Followers aayenge. Par ye ruthless hai. (fame +4, crush −2)</t>
         </is>
       </c>
       <c r="J30" s="2" t="n">
@@ -2565,12 +2569,12 @@
         <is>
           <t>ria: So this is who you are. Fine. You want my throne? You'll learn how heavy it is. This isn't over. 👑
 zoya: AND SCENE 💅✨ dekha babe? maine kaha tha. tune woh kiya jo mujhe karna tha — aur ilzaam tere sar. genius. 👀
-housewatch_india: NOT THE RECEIPTS 😭😭 ria's whole empire on borrowed money?? this house just went NUCLEAR #CreatorHouse #Exposed</t>
+House Watch: NOT THE RECEIPTS 😭😭 ria's whole empire on borrowed money?? this house just went NUCLEAR #CreatorHouse #Exposed</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>House Watch: the house is at WAR 🍿 team-exposed vs team-ria… iske baad koi normal nahi reh sakta. dropping everything to watch this 👀🔥 #CreatorHouse #Receipts</t>
+          <t>House Watch: the house is at WAR 🍿 team-exposed vs team-ria… iske baad koi normal nahi reh sakta 👀🔥 #CreatorHouse #Receipts</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2611,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Zoya ke khel mein haath mat daalo. Reach kam, dignity poori.</t>
+          <t>Zoya ke khel mein haath mat daalo. Reach kam, dignity poori. (fame −1, ally +3)</t>
         </is>
       </c>
       <c r="J31" s="2" t="n">
@@ -2626,37 +2630,169 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>kabir → Bhai maine dekha Zoya kya bhej rahi thi. Poora ghar us folder ka wait kar raha tha. 😳 / Aur tune delete kar diya. Ria ne tere saath kabhi seedha nahi kiya — tere haath mein usse barbaad karne ka mauka tha, aur tune nahi liya. / Followers baad mein bhi aa jaayenge yaar. Par jo tu aaj raat tha — woh Zoya kabhi nahi ban sakti. Main tujhe iske liye respect karta hoon. Sach. 🔥</t>
+          <t>kabir → Bhai maine dekha Zoya kya bhej rahi thi. Poora ghar us folder ka wait kar raha tha. 😳 / Aur tune delete kar diya. Ria ne tere saath kabhi seedha nahi kiya — tere haath mein usse barbaad karne ka mauka tha, aur tune nahi liya. / Followers baad mein bhi aa jaayenge yaar. Par jo tu aaj raat tha — woh Zoya kabhi nahi ban sakti. Main tujhe respect karta hoon. Sach. 🔥</t>
         </is>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
       <c r="Q31" s="2" t="inlineStr">
         <is>
-          <t>ria: Someone had my life in their hands last night. They chose to walk away clean. I don't forget things like that. Neither the kindness, nor the fact that they could. 🤍 #CreatorHouse</t>
+          <t>ria: Someone had my life in their hands last night. They chose to walk away clean. I don't forget things like that. 🤍 #CreatorHouse</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Very Late</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>D4-3</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Ria, Bina Mask  ⑂ {"flag": {"key": "allyEvicted", "gte": 1}}</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Ria ka sach — expose karoge, ya clean rahoge?</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Expose karo — sach post kar do</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Ria ka mask utaar do. Followers aayenge. Par ye ruthless hai. (fame +4, crush −2)</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>ananya −2</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr"/>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr"/>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>Is ghar mein sabke 'aesthetic' ke peeche kuch aur hota hai. Aaj kuch cheezein sabke saamne rakhta hoon. Truth over image. 👀 #CreatorHouse #Receipts</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>ria: So this is who you are. Fine. You want my throne? You'll learn how heavy it is. 👑
+zoya: AND SCENE 💅✨ tune woh kiya jo mujhe karna tha — aur ilzaam tere sar. genius. 👀
+House Watch: NOT THE RECEIPTS 😭😭 this house just went NUCLEAR #CreatorHouse #Exposed</t>
+        </is>
+      </c>
+      <c r="Q32" s="2" t="inlineStr">
+        <is>
+          <t>House Watch: the house is at WAR 🍿 team-exposed vs team-ria… iske baad koi normal nahi reh sakta 👀🔥 #CreatorHouse #Receipts</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Very Late</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>D4-3</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Ria, Bina Mask  ⑂ {"flag": {"key": "allyEvicted", "gte": 1}}</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Clean raho — screenshots delete karo</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Zoya ke khel mein haath mat daalo. Reach kam, dignity poori. (fame −1)</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>kabir → (bahar se, voice note) Bhai yahin baithe dekha — Zoya ne folder daala tha. 😳 / Aur tune delete kar diya. Followers chhod diye, izzat rakhi. Ghar se bahar hoke bhi keh raha hoon — tu wahi banda hai. / Jeet ke aana. Mere liye bhi. 🔥</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr"/>
+      <c r="P33" s="2" t="inlineStr"/>
+      <c r="Q33" s="2" t="inlineStr">
+        <is>
+          <t>ria: Someone had my life in their hands last night. They chose to walk away clean. I don't forget things like that. 🤍 #CreatorHouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Late Night</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>D5-1</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Aakhri Bada Faisla</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Late night. Villa chup hai. Finale ko chaubees ghante bhi nahi bache. House ka aakhri content window abhi khula hai — ek slot, prime time, saara internet online.
 Ek clean winner move ready hai — sirf tum, top pe, spotlight full. Numbers isse pyaar karenge. Bas Ananya ko frame ke bahar rakhna padega. Sab ke saamne.
@@ -2665,193 +2801,56 @@
 » Ye wahi sawaal hai jo Day 1 se chhupa tha — followers, ya feeling? Aaj raat jhooth nahi chalega.</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Aakhri raat — play to win, ya play for the romance?</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>Play to WIN</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>Winner move post karo. Spotlight sirf tumhara.</t>
         </is>
       </c>
-      <c r="J32" s="2" t="n">
+      <c r="J34" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="K32" s="2" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>ananya −4</t>
         </is>
       </c>
-      <c r="L32" s="2" t="inlineStr"/>
-      <c r="M32" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>Post</t>
         </is>
       </c>
-      <c r="N32" s="2" t="inlineStr"/>
-      <c r="O32" s="2" t="inlineStr">
+      <c r="N34" s="2" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr">
         <is>
           <t>Das din. Ek ghar. Aur main abhi bhi khada hoon — akela, apne dum pe. Kal finale. Baaki sab noise hai. 🏆 #CreatorHouse #FinaleEve</t>
         </is>
       </c>
-      <c r="P32" s="2" t="inlineStr">
+      <c r="P34" s="2" t="inlineStr">
         <is>
           <t>ria: Finale se ek raat pehle solo flex. Cold. Smart. Yahi to game hai. 👑
 ananya: Frame me jagah nahi thi na meri. Samajh gayi. Koi baat nahi. 🙂
 HouseWatch India: FINALE EVE aur ye banda solo chala gaya 👀 numbers ke liye sab chhod diya. iconic ya ice-cold? #CreatorHouse</t>
         </is>
       </c>
-      <c r="Q32" s="2" t="inlineStr">
+      <c r="Q34" s="2" t="inlineStr">
         <is>
           <t>HouseWatch India: Finale eve aur koi prime slot me akela chamak raha hai — apne closest bond ko frame se bahar rakhke. Numbers up. Dil ka pata nahi. 👀🏆 #CreatorHouse #Day5</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Late Night</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>D5-1</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Aakhri Bada Faisla</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr"/>
-      <c r="F33" s="2" t="inlineStr"/>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>Play for the ROMANCE</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>Slot chhodo. Aaj raat Ananya ke saath, camera ke bina.</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="n">
-        <v>-4</v>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>ananya +6</t>
-        </is>
-      </c>
-      <c r="L33" s="2" t="inlineStr"/>
-      <c r="M33" s="2" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="N33" s="2" t="inlineStr">
-        <is>
-          <t>ananya → Ruko… tumne prime slot chhod diya? Finale se ek raat pehle? 🥺 / Numbers ke liye nahi… mere liye? Sach me? / Chalo terrace pe. Camera band. Aaj raat sirf hum do. Ye… ye maine kabhi kisi ke saath feel nahi kiya. 🌙</t>
-        </is>
-      </c>
-      <c r="O33" s="2" t="inlineStr"/>
-      <c r="P33" s="2" t="inlineStr"/>
-      <c r="Q33" s="2" t="inlineStr">
-        <is>
-          <t>ananya: Kisi ne aaj raat pachaas hazaar log chhod diye… ek insaan ke liye. Main. 🌙 Kal jo bhi ho, ye raat meri hai. #FinaleEve</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Finale</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>D5-2</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Live Finale</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Live finale. Studio lights, 1.1 lakh log online. Stage pe Ria, Kabir, Ananya — sab bach gaye, sab tumhare saath khade hain.
-Host: Aur is season ka winner… hai… ye naam. Congratulations. Stage tumhara hai. 🎤
-Taaliyan. Camera tumhare chehre pe zoom hota hai. Kabir ki aankhein bhar aayi. Ananya bas dekh raha hai — jaise sab kuch is ek pal ka tha.
-» Das din. Ek mic. Ab jo bologe — wahi log yaad rakhenge. Ye tumhara hai. Kaise lete ho?</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>Result aa gaya — ise kaise lete ho?</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>Own it</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>Ye tumne kamaaya. Poora malik banke lo.</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>ananya +1, kabir +1</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr"/>
-      <c r="M34" s="2" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="N34" s="2" t="inlineStr">
-        <is>
-          <t>kabir → OYE WINNER 😭🔥 stage pe aise khada tha jaise ghar tera hi tha. mereko pata tha bhai. / haq se liya tune. koi begging nahi. that's my banda. 🔥 / Tumne ise apna banake liya. 🥺 Aur mujhe khushi hai maine tumhe uss raat dekha tha — before everyone else.</t>
-        </is>
-      </c>
-      <c r="O34" s="2" t="inlineStr"/>
-      <c r="P34" s="2" t="inlineStr"/>
-      <c r="Q34" s="2" t="inlineStr">
-        <is>
-          <t>HouseWatch India: AUR WINNER HAI… 🏆 stage pe aisa control jaise trophy pehle se hi inki thi. no shaking, no begging. season over. main character confirmed. 👑 #CreatorHouse #Finale</t>
         </is>
       </c>
     </row>
@@ -2861,17 +2860,17 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Finale</t>
+          <t>Late Night</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>D5-2</t>
+          <t>D5-1</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Live Finale</t>
+          <t>Aakhri Bada Faisla</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr"/>
@@ -2883,20 +2882,20 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Grateful / humble</t>
+          <t>Play for the ROMANCE</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Ye akele ka nahi tha. Sab ko lekar lo.</t>
+          <t>Slot chhodo. Aaj raat Ananya ke saath, camera ke bina.</t>
         </is>
       </c>
       <c r="J35" s="2" t="n">
-        <v>2</v>
+        <v>-4</v>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>ananya +2, kabir +2</t>
+          <t>ananya +6</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr"/>
@@ -2907,14 +2906,288 @@
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>kabir → bhai stage pe humaara naam liya tune 😭 sabke saamne. main ro diya lowkey. / trophy teri, par tune usko sabki bana diya. that's why tu jeeta. 🔥 / Tumne mujhe apne moment me kheencha. 🥺 Winner ho tum — par insaan pehle. Yahi yaad rahega mujhe.</t>
+          <t>ananya → Ruko… tumne prime slot chhod diya? Finale se ek raat pehle? 🥺 / Numbers ke liye nahi… mere liye? Sach me? / Chalo terrace pe. Camera band. Aaj raat sirf hum do. Ye… ye maine kabhi kisi ke saath feel nahi kiya. 🌙</t>
         </is>
       </c>
       <c r="O35" s="2" t="inlineStr"/>
       <c r="P35" s="2" t="inlineStr"/>
       <c r="Q35" s="2" t="inlineStr">
         <is>
-          <t>kabir: mera banda jeet gaya 😭🔥 aur trophy uthake sabse pehle humaara naam liya. yahi banda tha jo jeetne ke laayak tha. #Finale #CreatorHouse</t>
+          <t>ananya: Kisi ne aaj raat pachaas hazaar log chhod diye… ek insaan ke liye. Main. 🌙 Kal jo bhi ho, ye raat meri hai. #FinaleEve</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Finale</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>D5-2</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Live Finale</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Live finale. Studio lights, 1.1 lakh log online. Stage pe Ria, Kabir, Ananya — sab bach gaye, sab tumhare saath khade hain.
+Host: Aur is season ka winner… hai… ye naam. Congratulations. Stage tumhara hai. 🎤
+Taaliyan. Camera tumhare chehre pe zoom hota hai. Kabir ki aankhein bhar aayi. Ananya bas dekh rahi hai — jaise sab kuch is ek pal ka tha.
+» Das din. Ek mic. Ab jo bologe — wahi log yaad rakhenge. Ye tumhara hai. Kaise lete ho?</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Result aa gaya — ise kaise lete ho?</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Own it</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Ye tumne kamaaya. Poora malik banke lo.</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>ananya +1, kabir +1</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>kabir → OYE WINNER 😭🔥 stage pe aise khada tha jaise ghar tera hi tha. mereko pata tha bhai. / haq se liya tune. koi begging nahi. that's my banda. 🔥 / Tumne ise apna banake liya. 🥺 Aur mujhe khushi hai maine tumhe uss raat dekha tha — before everyone else.</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr"/>
+      <c r="P36" s="2" t="inlineStr"/>
+      <c r="Q36" s="2" t="inlineStr">
+        <is>
+          <t>HouseWatch India: AUR WINNER HAI… 🏆 stage pe aisa control jaise trophy pehle se hi inki thi. season over. main character confirmed. 👑 #CreatorHouse #Finale</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Finale</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>D5-2</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Live Finale</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Grateful / humble</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Ye akele ka nahi tha. Sab ko lekar lo.</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>ananya +2, kabir +2</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr"/>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>kabir → bhai stage pe humaara naam liya tune 😭 sabke saamne. main ro diya lowkey. / trophy teri, par tune usko sabki bana diya. that's why tu jeeta. 🔥 / Tumne mujhe apne moment me kheencha. 🥺 Winner ho tum — par insaan pehle. Yahi yaad rahega mujhe.</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr"/>
+      <c r="P37" s="2" t="inlineStr"/>
+      <c r="Q37" s="2" t="inlineStr">
+        <is>
+          <t>kabir: mera banda jeet gaya 😭🔥 aur trophy uthake sabse pehle humaara naam liya. yahi banda jeetne ke laayak tha. #Finale #CreatorHouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Finale</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>D5-2</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Live Finale  ⑂ {"flag": {"key": "allyEvicted", "gte": 1}}</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Live finale. Studio lights, 1.1 lakh log online. Stage pe Ria aur Ananya — Kabir is safar mein aakhir tak nahi pahuncha, par uski jagah tum aaj bhi mehsoos karte ho.
+Host: Aur is season ka winner… hai… ye naam. Congratulations. Stage tumhara hai. 🎤
+Taaliyan. Ananya ki aankhein bhar aayi — woh dekh rahi hai jaise sab kuch is ek pal ka tha.
+» Das din. Ek mic. Ye tumhara hai. Kaise lete ho?</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Result aa gaya — ise kaise lete ho?</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Own it</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Ye tumne kamaaya. Poora malik banke lo.</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>ananya +1</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>ananya → Tumne ise apna banake liya. 🥺 Aur main? Maine tumhe uss raat dekha tha — before everyone else. / (bahar se) OYE WINNER 😭🔥 ghar se nikal gaya par tujhe jeette dekh liya. haq se liya tune. that's my banda.</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr"/>
+      <c r="P38" s="2" t="inlineStr"/>
+      <c r="Q38" s="2" t="inlineStr">
+        <is>
+          <t>HouseWatch India: AUR WINNER HAI… 🏆 stage pe aisa control jaise trophy pehle se hi inki thi. season over. main character confirmed. 👑 #CreatorHouse #Finale</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Finale</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>D5-2</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Live Finale  ⑂ {"flag": {"key": "allyEvicted", "gte": 1}}</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr"/>
+      <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Grateful / humble</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Ye akele ka nahi tha. Sab ko lekar lo.</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>ananya +2</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>ananya → Tumne mujhe apne moment me kheencha. 🥺 Winner ho tum — par insaan pehle. Yahi yaad rahega mujhe. / (bahar se) bhai stage pe humaara naam liya tune 😭 main bahar se ro diya. that's why tu jeeta.</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr"/>
+      <c r="P39" s="2" t="inlineStr"/>
+      <c r="Q39" s="2" t="inlineStr">
+        <is>
+          <t>kabir: mera banda jeet gaya 😭🔥 aur trophy uthake sabse pehle humaara naam liya. yahi banda jeetne ke laayak tha. #Finale #CreatorHouse</t>
         </is>
       </c>
     </row>
@@ -3230,7 +3503,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>16 beats. Source: public/content/creator-house-v4.json (version 8).</t>
+          <t>16 beats. Source: public/content/creator-house-v4.json (version 9).</t>
         </is>
       </c>
     </row>

</xml_diff>